<commit_message>
agentic-qe-mvp: static header; Test data agent as the eighth core agent
Co-Authored-By: Devin AI <158243242+devin-ai-integration[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/agentic-qe-mvp/demo-artifacts/flow-1-baseline-CYC-1/04-test-cases/CYC-1-test-cases.xlsx
+++ b/agentic-qe-mvp/demo-artifacts/flow-1-baseline-CYC-1/04-test-cases/CYC-1-test-cases.xlsx
@@ -5,14 +5,15 @@
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
     <sheet sheetId="1" name="Test Cases" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="About" state="visible" r:id="rId5"/>
+    <sheet sheetId="2" name="Test Data" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="About" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="387" uniqueCount="212">
   <si>
     <t>Key</t>
   </si>
@@ -478,6 +479,250 @@
     <t>README.md, REQ-014, BR-014</t>
   </si>
   <si>
+    <t>Data Set</t>
+  </si>
+  <si>
+    <t>Test Case</t>
+  </si>
+  <si>
+    <t>Requirement</t>
+  </si>
+  <si>
+    <t>Set By Test Case</t>
+  </si>
+  <si>
+    <t>Generated From Spec</t>
+  </si>
+  <si>
+    <t>Check Against Spec</t>
+  </si>
+  <si>
+    <t>Problems</t>
+  </si>
+  <si>
+    <t>Version</t>
+  </si>
+  <si>
+    <t>TD-F-001</t>
+  </si>
+  <si>
+    <t>REQ-001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">reservation.status = CONFIRMED
+channel.bookingChannel = DIRECT
+stay.nights = 3
+rate.planCategory = BAR
+room.roomCount = 1
+payment.loyaltyPointsRedemption = false
+revenue.totalAmount = 1000
+revenue.taxAmount = 120
+revenue.resortFeeAmount = 30
+revenue.ancillaryAmount = 50</t>
+  </si>
+  <si>
+    <t>990 attributes</t>
+  </si>
+  <si>
+    <t>conforms</t>
+  </si>
+  <si>
+    <t>new</t>
+  </si>
+  <si>
+    <t>TD-F-002</t>
+  </si>
+  <si>
+    <t>REQ-002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">reservation.status = CONFIRMED
+channel.bookingChannel = GDS
+stay.nights = 3
+rate.planCategory = BAR
+room.roomCount = 1
+payment.loyaltyPointsRedemption = false
+revenue.totalAmount = 1000
+revenue.taxAmount = 120
+revenue.resortFeeAmount = 30
+revenue.ancillaryAmount = 50</t>
+  </si>
+  <si>
+    <t>TD-N-001</t>
+  </si>
+  <si>
+    <t>REQ-003</t>
+  </si>
+  <si>
+    <t>TD-F-003</t>
+  </si>
+  <si>
+    <t>REQ-004</t>
+  </si>
+  <si>
+    <t>TD-F-004</t>
+  </si>
+  <si>
+    <t>REQ-005</t>
+  </si>
+  <si>
+    <t>TD-F-005</t>
+  </si>
+  <si>
+    <t>REQ-006</t>
+  </si>
+  <si>
+    <t>TD-F-006</t>
+  </si>
+  <si>
+    <t>REQ-007</t>
+  </si>
+  <si>
+    <t xml:space="preserve">reservation.status = CONFIRMED
+channel.bookingChannel = DIRECT
+stay.nights = 7
+rate.planCategory = BAR
+room.roomCount = 1
+payment.loyaltyPointsRedemption = false
+revenue.totalAmount = 1000
+revenue.taxAmount = 120
+revenue.resortFeeAmount = 30
+revenue.ancillaryAmount = 50</t>
+  </si>
+  <si>
+    <t>TD-F-007</t>
+  </si>
+  <si>
+    <t xml:space="preserve">reservation.status = CONFIRMED
+channel.bookingChannel = DIRECT
+stay.nights = 6
+rate.planCategory = BAR
+room.roomCount = 1
+payment.loyaltyPointsRedemption = false
+revenue.totalAmount = 1000
+revenue.taxAmount = 120
+revenue.resortFeeAmount = 30
+revenue.ancillaryAmount = 50</t>
+  </si>
+  <si>
+    <t>TD-F-008</t>
+  </si>
+  <si>
+    <t>REQ-008</t>
+  </si>
+  <si>
+    <t xml:space="preserve">reservation.status = CONFIRMED
+channel.bookingChannel = DIRECT
+stay.nights = 3
+rate.planCategory = BAR
+room.roomCount = 1
+payment.loyaltyPointsRedemption = false
+revenue.totalAmount = 8000
+revenue.taxAmount = 0
+revenue.resortFeeAmount = 0
+revenue.ancillaryAmount = 0</t>
+  </si>
+  <si>
+    <t>TD-F-009</t>
+  </si>
+  <si>
+    <t>REQ-009</t>
+  </si>
+  <si>
+    <t xml:space="preserve">reservation.status = CONFIRMED
+channel.bookingChannel = DIRECT
+stay.nights = 3
+rate.planCategory = BAR
+room.roomCount = 1
+payment.loyaltyPointsRedemption = false
+revenue.totalAmount = 123.45
+revenue.taxAmount = 0
+revenue.resortFeeAmount = 0
+revenue.ancillaryAmount = 0</t>
+  </si>
+  <si>
+    <t>TD-F-010</t>
+  </si>
+  <si>
+    <t>REQ-010</t>
+  </si>
+  <si>
+    <t xml:space="preserve">reservation.status = CONFIRMED
+channel.bookingChannel = DIRECT
+stay.nights = 3
+rate.planCategory = BAR
+room.roomCount = 1
+payment.loyaltyPointsRedemption = true
+revenue.totalAmount = 1000
+revenue.taxAmount = 120
+revenue.resortFeeAmount = 30
+revenue.ancillaryAmount = 50</t>
+  </si>
+  <si>
+    <t>TD-F-011</t>
+  </si>
+  <si>
+    <t>REQ-011</t>
+  </si>
+  <si>
+    <t xml:space="preserve">reservation.status = CANCELLED | NO_SHOW
+channel.bookingChannel = DIRECT
+stay.nights = 3
+rate.planCategory = BAR
+room.roomCount = 1
+payment.loyaltyPointsRedemption = false
+revenue.totalAmount = 1000
+revenue.taxAmount = 120
+revenue.resortFeeAmount = 30
+revenue.ancillaryAmount = 50</t>
+  </si>
+  <si>
+    <t>TD-F-012</t>
+  </si>
+  <si>
+    <t>REQ-012</t>
+  </si>
+  <si>
+    <t>standard booking</t>
+  </si>
+  <si>
+    <t>1000 attributes</t>
+  </si>
+  <si>
+    <t>TD-F-013</t>
+  </si>
+  <si>
+    <t>REQ-013</t>
+  </si>
+  <si>
+    <t xml:space="preserve">reservation.status = CONFIRMED
+channel.bookingChannel = DIRECT
+stay.nights = 3
+rate.planCategory = BAR
+room.roomCount = 1
+payment.loyaltyPointsRedemption = false
+revenue.totalAmount = 1000
+revenue.taxAmount = 120
+revenue.resortFeeAmount = 30
+revenue.ancillaryAmount = 50
+advisor.iataNumber = </t>
+  </si>
+  <si>
+    <t>989 attributes</t>
+  </si>
+  <si>
+    <t>negative test</t>
+  </si>
+  <si>
+    <t>advisor.iataNumber is required but empty</t>
+  </si>
+  <si>
+    <t>TD-F-014</t>
+  </si>
+  <si>
+    <t>REQ-014</t>
+  </si>
+  <si>
     <t>Field</t>
   </si>
   <si>
@@ -499,7 +744,7 @@
     <t>Exported at</t>
   </si>
   <si>
-    <t>2026-09-29T17:20:33.063Z</t>
+    <t>2026-09-29T19:40:18.420Z</t>
   </si>
   <si>
     <t>Column order</t>
@@ -1693,6 +1938,489 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:I16"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="3" width="12" customWidth="1"/>
+    <col min="4" max="4" width="48" customWidth="1"/>
+    <col min="5" max="5" width="20" customWidth="1"/>
+    <col min="6" max="6" width="18" customWidth="1"/>
+    <col min="7" max="7" width="40" customWidth="1"/>
+    <col min="8" max="8" width="14" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="I2" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="I3" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="I4" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="I5" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="I6" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="I7" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="I8" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="I9" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="I10" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="I11" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="I12" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="I13" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="I14" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="I15" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="I16" s="2">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
@@ -1702,18 +2430,18 @@
   <sheetData>
     <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>142</v>
+        <v>196</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>143</v>
+        <v>197</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>144</v>
+        <v>198</v>
       </c>
       <c r="B2" t="s">
-        <v>145</v>
+        <v>199</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -1721,7 +2449,7 @@
         <v>12</v>
       </c>
       <c r="B3" t="s">
-        <v>146</v>
+        <v>200</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -1729,47 +2457,47 @@
         <v>28</v>
       </c>
       <c r="B4" t="s">
-        <v>147</v>
+        <v>201</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>148</v>
+        <v>202</v>
       </c>
       <c r="B5" t="s">
-        <v>149</v>
+        <v>203</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>150</v>
+        <v>204</v>
       </c>
       <c r="B6" t="s">
-        <v>151</v>
+        <v>205</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>152</v>
+        <v>206</v>
       </c>
       <c r="B7" t="s">
-        <v>153</v>
+        <v>207</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>154</v>
+        <v>208</v>
       </c>
       <c r="B8" t="s">
-        <v>155</v>
+        <v>209</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>156</v>
+        <v>210</v>
       </c>
       <c r="B9" t="s">
-        <v>157</v>
+        <v>211</v>
       </c>
     </row>
   </sheetData>

</xml_diff>